<commit_message>
Add refrigeration output variables
</commit_message>
<xml_diff>
--- a/measures/comstock_sensitivity_reports/resources/Variable List.xlsx
+++ b/measures/comstock_sensitivity_reports/resources/Variable List.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccaradon\Documents\GitHub\ComStock\measures\comstock_sensitivity_reports\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mdahlhau\Documents\GitHub\NREL\comstock\measures\comstock_sensitivity_reports\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D0781B6-2CFF-43BC-A295-C8D9EBDAEB0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEACB07F-5581-4FD3-92BA-A54C6C03D12F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="672" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{35549412-5E91-4CB3-A95B-F037AB4A5442}"/>
+    <workbookView xWindow="1830" yWindow="495" windowWidth="26340" windowHeight="14070" firstSheet="1" activeTab="1" xr2:uid="{35549412-5E91-4CB3-A95B-F037AB4A5442}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="hidden" r:id="rId1"/>
@@ -45,7 +45,7 @@
     <author>tc={41EBC68D-AB6D-4CC4-A69A-78845442F100}</author>
   </authors>
   <commentList>
-    <comment ref="F353" authorId="0" shapeId="0" xr:uid="{41EBC68D-AB6D-4CC4-A69A-78845442F100}">
+    <comment ref="F357" authorId="0" shapeId="0" xr:uid="{41EBC68D-AB6D-4CC4-A69A-78845442F100}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3108" uniqueCount="991">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3136" uniqueCount="999">
   <si>
     <t>Input List</t>
   </si>
@@ -3031,6 +3031,30 @@
   </si>
   <si>
     <t>air_system_vav_avg_flow_ratio</t>
+  </si>
+  <si>
+    <t>com_report_refrigeration_case_count</t>
+  </si>
+  <si>
+    <t>com_report_refrigeration_case_total_defrost_electric_j</t>
+  </si>
+  <si>
+    <t>com_report_refrigeration_walk_in_count</t>
+  </si>
+  <si>
+    <t>com_report_refrigeration_walk_in_total_defrost_electric_j</t>
+  </si>
+  <si>
+    <t>Refrigeration case count</t>
+  </si>
+  <si>
+    <t>Refrigeration walk-in count</t>
+  </si>
+  <si>
+    <t>Refrigeration walk-in defrost energy</t>
+  </si>
+  <si>
+    <t>Refrigeration case defrost energy</t>
   </si>
 </sst>
 </file>
@@ -3114,20 +3138,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor theme="6"/>
         </patternFill>
       </fill>
@@ -3185,6 +3195,20 @@
       <fill>
         <patternFill>
           <bgColor theme="6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3560,7 +3584,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="F353" dT="2025-10-30T14:26:48.21" personId="{77426C77-5C18-4B27-8B0E-67F1F50A374F}" id="{41EBC68D-AB6D-4CC4-A69A-78845442F100}">
+  <threadedComment ref="F357" dT="2025-10-30T14:26:48.21" personId="{77426C77-5C18-4B27-8B0E-67F1F50A374F}" id="{41EBC68D-AB6D-4CC4-A69A-78845442F100}">
     <text>Output is boolean; do we need a converter?</text>
   </threadedComment>
 </ThreadedComments>
@@ -4924,7 +4948,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CE568D5-2279-4922-8B77-550F2E5B90B6}">
-  <dimension ref="A1:K357"/>
+  <dimension ref="A1:K361"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="64.7109375" bestFit="1" customWidth="1"/>
@@ -13547,13 +13571,19 @@
     </row>
     <row r="342" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
-        <v>925</v>
+        <v>995</v>
       </c>
       <c r="B342" t="s">
-        <v>106</v>
+        <v>133</v>
       </c>
       <c r="D342" t="s">
-        <v>926</v>
+        <v>991</v>
+      </c>
+      <c r="E342" t="s">
+        <v>152</v>
+      </c>
+      <c r="F342" t="s">
+        <v>141</v>
       </c>
       <c r="H342" t="s">
         <v>119</v>
@@ -13564,13 +13594,19 @@
     </row>
     <row r="343" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
-        <v>927</v>
+        <v>998</v>
       </c>
       <c r="B343" t="s">
-        <v>106</v>
+        <v>133</v>
       </c>
       <c r="D343" t="s">
-        <v>928</v>
+        <v>992</v>
+      </c>
+      <c r="E343" t="s">
+        <v>152</v>
+      </c>
+      <c r="F343" t="s">
+        <v>141</v>
       </c>
       <c r="H343" t="s">
         <v>119</v>
@@ -13581,13 +13617,19 @@
     </row>
     <row r="344" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
-        <v>972</v>
+        <v>996</v>
       </c>
       <c r="B344" t="s">
-        <v>970</v>
+        <v>133</v>
       </c>
       <c r="D344" t="s">
-        <v>961</v>
+        <v>993</v>
+      </c>
+      <c r="E344" t="s">
+        <v>152</v>
+      </c>
+      <c r="F344" t="s">
+        <v>141</v>
       </c>
       <c r="H344" t="s">
         <v>119</v>
@@ -13598,13 +13640,19 @@
     </row>
     <row r="345" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
-        <v>971</v>
+        <v>997</v>
       </c>
       <c r="B345" t="s">
-        <v>970</v>
+        <v>133</v>
       </c>
       <c r="D345" t="s">
-        <v>962</v>
+        <v>994</v>
+      </c>
+      <c r="E345" t="s">
+        <v>152</v>
+      </c>
+      <c r="F345" t="s">
+        <v>141</v>
       </c>
       <c r="H345" t="s">
         <v>119</v>
@@ -13615,13 +13663,13 @@
     </row>
     <row r="346" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
-        <v>973</v>
+        <v>925</v>
       </c>
       <c r="B346" t="s">
-        <v>970</v>
+        <v>106</v>
       </c>
       <c r="D346" t="s">
-        <v>963</v>
+        <v>926</v>
       </c>
       <c r="H346" t="s">
         <v>119</v>
@@ -13632,13 +13680,13 @@
     </row>
     <row r="347" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
-        <v>974</v>
+        <v>927</v>
       </c>
       <c r="B347" t="s">
-        <v>970</v>
+        <v>106</v>
       </c>
       <c r="D347" t="s">
-        <v>964</v>
+        <v>928</v>
       </c>
       <c r="H347" t="s">
         <v>119</v>
@@ -13649,13 +13697,13 @@
     </row>
     <row r="348" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
-        <v>975</v>
+        <v>972</v>
       </c>
       <c r="B348" t="s">
         <v>970</v>
       </c>
       <c r="D348" t="s">
-        <v>965</v>
+        <v>961</v>
       </c>
       <c r="H348" t="s">
         <v>119</v>
@@ -13666,13 +13714,13 @@
     </row>
     <row r="349" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
-        <v>976</v>
+        <v>971</v>
       </c>
       <c r="B349" t="s">
         <v>970</v>
       </c>
       <c r="D349" t="s">
-        <v>966</v>
+        <v>962</v>
       </c>
       <c r="H349" t="s">
         <v>119</v>
@@ -13683,13 +13731,13 @@
     </row>
     <row r="350" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
-        <v>977</v>
+        <v>973</v>
       </c>
       <c r="B350" t="s">
         <v>970</v>
       </c>
       <c r="D350" t="s">
-        <v>967</v>
+        <v>963</v>
       </c>
       <c r="H350" t="s">
         <v>119</v>
@@ -13700,13 +13748,13 @@
     </row>
     <row r="351" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
-        <v>978</v>
+        <v>974</v>
       </c>
       <c r="B351" t="s">
         <v>970</v>
       </c>
       <c r="D351" t="s">
-        <v>968</v>
+        <v>964</v>
       </c>
       <c r="H351" t="s">
         <v>119</v>
@@ -13717,13 +13765,13 @@
     </row>
     <row r="352" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
-        <v>979</v>
+        <v>975</v>
       </c>
       <c r="B352" t="s">
         <v>970</v>
       </c>
       <c r="D352" t="s">
-        <v>969</v>
+        <v>965</v>
       </c>
       <c r="H352" t="s">
         <v>119</v>
@@ -13734,104 +13782,172 @@
     </row>
     <row r="353" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
-        <v>980</v>
+        <v>976</v>
       </c>
       <c r="B353" t="s">
-        <v>106</v>
+        <v>970</v>
       </c>
       <c r="D353" t="s">
-        <v>981</v>
-      </c>
-      <c r="E353" t="s">
-        <v>152</v>
-      </c>
-      <c r="F353" t="s">
-        <v>982</v>
+        <v>966</v>
       </c>
       <c r="H353" t="s">
+        <v>119</v>
+      </c>
+      <c r="I353" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="354" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
-        <v>983</v>
+        <v>977</v>
       </c>
       <c r="B354" t="s">
-        <v>106</v>
+        <v>970</v>
       </c>
       <c r="D354" t="s">
-        <v>984</v>
-      </c>
-      <c r="E354" t="s">
-        <v>152</v>
-      </c>
-      <c r="F354" t="s">
-        <v>982</v>
+        <v>967</v>
       </c>
       <c r="H354" t="s">
+        <v>119</v>
+      </c>
+      <c r="I354" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="355" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
-        <v>985</v>
+        <v>978</v>
       </c>
       <c r="B355" t="s">
-        <v>106</v>
+        <v>970</v>
       </c>
       <c r="D355" t="s">
-        <v>986</v>
-      </c>
-      <c r="E355" t="s">
-        <v>152</v>
-      </c>
-      <c r="F355" t="s">
-        <v>982</v>
+        <v>968</v>
       </c>
       <c r="H355" t="s">
+        <v>119</v>
+      </c>
+      <c r="I355" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="356" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
-        <v>987</v>
+        <v>979</v>
       </c>
       <c r="B356" t="s">
-        <v>106</v>
+        <v>970</v>
       </c>
       <c r="D356" t="s">
-        <v>988</v>
-      </c>
-      <c r="E356" t="s">
-        <v>152</v>
-      </c>
-      <c r="F356" t="s">
-        <v>982</v>
+        <v>969</v>
       </c>
       <c r="H356" t="s">
+        <v>119</v>
+      </c>
+      <c r="I356" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="357" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
+        <v>980</v>
+      </c>
+      <c r="B357" t="s">
+        <v>106</v>
+      </c>
+      <c r="D357" t="s">
+        <v>981</v>
+      </c>
+      <c r="E357" t="s">
+        <v>152</v>
+      </c>
+      <c r="F357" t="s">
+        <v>982</v>
+      </c>
+      <c r="H357" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="358" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A358" t="s">
+        <v>983</v>
+      </c>
+      <c r="B358" t="s">
+        <v>106</v>
+      </c>
+      <c r="D358" t="s">
+        <v>984</v>
+      </c>
+      <c r="E358" t="s">
+        <v>152</v>
+      </c>
+      <c r="F358" t="s">
+        <v>982</v>
+      </c>
+      <c r="H358" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="359" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A359" t="s">
+        <v>985</v>
+      </c>
+      <c r="B359" t="s">
+        <v>106</v>
+      </c>
+      <c r="D359" t="s">
+        <v>986</v>
+      </c>
+      <c r="E359" t="s">
+        <v>152</v>
+      </c>
+      <c r="F359" t="s">
+        <v>982</v>
+      </c>
+      <c r="H359" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="360" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A360" t="s">
+        <v>987</v>
+      </c>
+      <c r="B360" t="s">
+        <v>106</v>
+      </c>
+      <c r="D360" t="s">
+        <v>988</v>
+      </c>
+      <c r="E360" t="s">
+        <v>152</v>
+      </c>
+      <c r="F360" t="s">
+        <v>982</v>
+      </c>
+      <c r="H360" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="361" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A361" t="s">
         <v>989</v>
       </c>
-      <c r="B357" t="s">
-        <v>106</v>
-      </c>
-      <c r="D357" t="s">
+      <c r="B361" t="s">
+        <v>106</v>
+      </c>
+      <c r="D361" t="s">
         <v>990</v>
       </c>
-      <c r="E357" t="s">
-        <v>152</v>
-      </c>
-      <c r="F357" t="s">
-        <v>141</v>
-      </c>
-      <c r="H357" t="s">
-        <v>119</v>
-      </c>
-      <c r="I357" t="s">
+      <c r="E361" t="s">
+        <v>152</v>
+      </c>
+      <c r="F361" t="s">
+        <v>141</v>
+      </c>
+      <c r="H361" t="s">
+        <v>119</v>
+      </c>
+      <c r="I361" t="s">
         <v>119</v>
       </c>
     </row>
@@ -13841,7 +13957,7 @@
       <sortCondition ref="B1:B341"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="E2:E341 J16:J21 J86:J91 J105 J117 J149 J214">
+  <conditionalFormatting sqref="J16:J21 J86:J91 J105 J117 J149 J214 E2:E345">
     <cfRule type="containsText" dxfId="19" priority="90" operator="containsText" text="no">
       <formula>NOT(ISERROR(SEARCH("no",E2)))</formula>
     </cfRule>
@@ -13849,7 +13965,7 @@
       <formula>NOT(ISERROR(SEARCH("yes",E2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E341">
+  <conditionalFormatting sqref="E2:E345">
     <cfRule type="containsText" dxfId="17" priority="87" operator="containsText" text="no">
       <formula>NOT(ISERROR(SEARCH("no",E2)))</formula>
     </cfRule>
@@ -13857,68 +13973,64 @@
       <formula>NOT(ISERROR(SEARCH("TBD",E2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E353:F356">
-    <cfRule type="containsText" dxfId="15" priority="5" operator="containsText" text="no">
-      <formula>NOT(ISERROR(SEARCH("no",E353)))</formula>
+  <conditionalFormatting sqref="E361">
+    <cfRule type="containsText" dxfId="15" priority="1" operator="containsText" text="no">
+      <formula>NOT(ISERROR(SEARCH("no",E361)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="6" operator="containsText" text="TBD">
-      <formula>NOT(ISERROR(SEARCH("TBD",E353)))</formula>
+    <cfRule type="containsText" dxfId="14" priority="2" operator="containsText" text="TBD">
+      <formula>NOT(ISERROR(SEARCH("TBD",E361)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="7" operator="containsText" text="no">
-      <formula>NOT(ISERROR(SEARCH("no",E353)))</formula>
+    <cfRule type="containsText" dxfId="13" priority="3" operator="containsText" text="no">
+      <formula>NOT(ISERROR(SEARCH("no",E361)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="8" operator="containsText" text="yes">
-      <formula>NOT(ISERROR(SEARCH("yes",E353)))</formula>
+    <cfRule type="containsText" dxfId="12" priority="4" operator="containsText" text="yes">
+      <formula>NOT(ISERROR(SEARCH("yes",E361)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:I352">
-    <cfRule type="containsText" dxfId="11" priority="9" operator="containsText" text="no">
+  <conditionalFormatting sqref="E357:F360">
+    <cfRule type="containsText" dxfId="11" priority="5" operator="containsText" text="no">
+      <formula>NOT(ISERROR(SEARCH("no",E357)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="10" priority="6" operator="containsText" text="TBD">
+      <formula>NOT(ISERROR(SEARCH("TBD",E357)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="9" priority="7" operator="containsText" text="no">
+      <formula>NOT(ISERROR(SEARCH("no",E357)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="8" priority="8" operator="containsText" text="yes">
+      <formula>NOT(ISERROR(SEARCH("yes",E357)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:I356">
+    <cfRule type="containsText" dxfId="7" priority="9" operator="containsText" text="no">
       <formula>NOT(ISERROR(SEARCH("no",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="10" operator="containsText" text="yes">
+    <cfRule type="containsText" dxfId="6" priority="10" operator="containsText" text="yes">
       <formula>NOT(ISERROR(SEARCH("yes",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J152:J154">
-    <cfRule type="containsText" dxfId="9" priority="55" operator="containsText" text="no">
+    <cfRule type="containsText" dxfId="5" priority="55" operator="containsText" text="no">
       <formula>NOT(ISERROR(SEARCH("no",J152)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="56" operator="containsText" text="yes">
+    <cfRule type="containsText" dxfId="4" priority="56" operator="containsText" text="yes">
       <formula>NOT(ISERROR(SEARCH("yes",J152)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J157:J158">
-    <cfRule type="containsText" dxfId="7" priority="53" operator="containsText" text="no">
+    <cfRule type="containsText" dxfId="3" priority="53" operator="containsText" text="no">
       <formula>NOT(ISERROR(SEARCH("no",J157)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="54" operator="containsText" text="yes">
+    <cfRule type="containsText" dxfId="2" priority="54" operator="containsText" text="yes">
       <formula>NOT(ISERROR(SEARCH("yes",J157)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J225:J233">
-    <cfRule type="containsText" dxfId="5" priority="57" operator="containsText" text="no">
+    <cfRule type="containsText" dxfId="1" priority="57" operator="containsText" text="no">
       <formula>NOT(ISERROR(SEARCH("no",J225)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="58" operator="containsText" text="yes">
+    <cfRule type="containsText" dxfId="0" priority="58" operator="containsText" text="yes">
       <formula>NOT(ISERROR(SEARCH("yes",J225)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E357">
-    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="no">
-      <formula>NOT(ISERROR(SEARCH("no",E357)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E357">
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="no">
-      <formula>NOT(ISERROR(SEARCH("no",E357)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="TBD">
-      <formula>NOT(ISERROR(SEARCH("TBD",E357)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E357">
-    <cfRule type="containsText" dxfId="0" priority="4" operator="containsText" text="yes">
-      <formula>NOT(ISERROR(SEARCH("yes",E357)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
split out med and low temp defrost
</commit_message>
<xml_diff>
--- a/measures/comstock_sensitivity_reports/resources/Variable List.xlsx
+++ b/measures/comstock_sensitivity_reports/resources/Variable List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mdahlhau\Documents\GitHub\NREL\comstock\measures\comstock_sensitivity_reports\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEACB07F-5581-4FD3-92BA-A54C6C03D12F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDEC1AB0-91AD-4F93-AF79-21F8A8DFBA63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1830" yWindow="495" windowWidth="26340" windowHeight="14070" firstSheet="1" activeTab="1" xr2:uid="{35549412-5E91-4CB3-A95B-F037AB4A5442}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{35549412-5E91-4CB3-A95B-F037AB4A5442}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="hidden" r:id="rId1"/>
@@ -45,7 +45,7 @@
     <author>tc={41EBC68D-AB6D-4CC4-A69A-78845442F100}</author>
   </authors>
   <commentList>
-    <comment ref="F357" authorId="0" shapeId="0" xr:uid="{41EBC68D-AB6D-4CC4-A69A-78845442F100}">
+    <comment ref="F361" authorId="0" shapeId="0" xr:uid="{41EBC68D-AB6D-4CC4-A69A-78845442F100}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3136" uniqueCount="999">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3164" uniqueCount="1007">
   <si>
     <t>Input List</t>
   </si>
@@ -3033,28 +3033,52 @@
     <t>air_system_vav_avg_flow_ratio</t>
   </si>
   <si>
-    <t>com_report_refrigeration_case_count</t>
-  </si>
-  <si>
-    <t>com_report_refrigeration_case_total_defrost_electric_j</t>
-  </si>
-  <si>
-    <t>com_report_refrigeration_walk_in_count</t>
-  </si>
-  <si>
-    <t>com_report_refrigeration_walk_in_total_defrost_electric_j</t>
-  </si>
-  <si>
-    <t>Refrigeration case count</t>
-  </si>
-  <si>
-    <t>Refrigeration walk-in count</t>
-  </si>
-  <si>
-    <t>Refrigeration walk-in defrost energy</t>
-  </si>
-  <si>
-    <t>Refrigeration case defrost energy</t>
+    <t>com_report_refrigeration_med_temp_case_count</t>
+  </si>
+  <si>
+    <t>com_report_refrigeration_med_temp_case_total_defrost_electric_j</t>
+  </si>
+  <si>
+    <t>com_report_refrigeration_med_temp_walk_in_count</t>
+  </si>
+  <si>
+    <t>com_report_refrigeration_med_temp_walk_in_total_defrost_electric_j</t>
+  </si>
+  <si>
+    <t>com_report_refrigeration_low_temp_case_count</t>
+  </si>
+  <si>
+    <t>com_report_refrigeration_low_temp_case_total_defrost_electric_j</t>
+  </si>
+  <si>
+    <t>com_report_refrigeration_low_temp_walk_in_count</t>
+  </si>
+  <si>
+    <t>com_report_refrigeration_low_temp_walk_in_total_defrost_electric_j</t>
+  </si>
+  <si>
+    <t>Refrigeration med temp case count</t>
+  </si>
+  <si>
+    <t>Refrigeration med temp case defrost energy</t>
+  </si>
+  <si>
+    <t>Refrigeration med temp walk-in count</t>
+  </si>
+  <si>
+    <t>Refrigeration med temp walk-in defrost energy</t>
+  </si>
+  <si>
+    <t>Refrigeration low temp case count</t>
+  </si>
+  <si>
+    <t>Refrigeration low temp case defrost energy</t>
+  </si>
+  <si>
+    <t>Refrigeration low temp walk-in count</t>
+  </si>
+  <si>
+    <t>Refrigeration low temp walk-in defrost energy</t>
   </si>
 </sst>
 </file>
@@ -3584,7 +3608,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="F357" dT="2025-10-30T14:26:48.21" personId="{77426C77-5C18-4B27-8B0E-67F1F50A374F}" id="{41EBC68D-AB6D-4CC4-A69A-78845442F100}">
+  <threadedComment ref="F361" dT="2025-10-30T14:26:48.21" personId="{77426C77-5C18-4B27-8B0E-67F1F50A374F}" id="{41EBC68D-AB6D-4CC4-A69A-78845442F100}">
     <text>Output is boolean; do we need a converter?</text>
   </threadedComment>
 </ThreadedComments>
@@ -4948,7 +4972,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CE568D5-2279-4922-8B77-550F2E5B90B6}">
-  <dimension ref="A1:K361"/>
+  <dimension ref="A1:K365"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="64.7109375" bestFit="1" customWidth="1"/>
@@ -13571,7 +13595,7 @@
     </row>
     <row r="342" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
-        <v>995</v>
+        <v>999</v>
       </c>
       <c r="B342" t="s">
         <v>133</v>
@@ -13594,7 +13618,7 @@
     </row>
     <row r="343" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
-        <v>998</v>
+        <v>1000</v>
       </c>
       <c r="B343" t="s">
         <v>133</v>
@@ -13617,7 +13641,7 @@
     </row>
     <row r="344" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
-        <v>996</v>
+        <v>1001</v>
       </c>
       <c r="B344" t="s">
         <v>133</v>
@@ -13640,7 +13664,7 @@
     </row>
     <row r="345" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
-        <v>997</v>
+        <v>1002</v>
       </c>
       <c r="B345" t="s">
         <v>133</v>
@@ -13663,13 +13687,19 @@
     </row>
     <row r="346" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
-        <v>925</v>
+        <v>1003</v>
       </c>
       <c r="B346" t="s">
-        <v>106</v>
+        <v>133</v>
       </c>
       <c r="D346" t="s">
-        <v>926</v>
+        <v>995</v>
+      </c>
+      <c r="E346" t="s">
+        <v>152</v>
+      </c>
+      <c r="F346" t="s">
+        <v>141</v>
       </c>
       <c r="H346" t="s">
         <v>119</v>
@@ -13680,13 +13710,19 @@
     </row>
     <row r="347" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
-        <v>927</v>
+        <v>1004</v>
       </c>
       <c r="B347" t="s">
-        <v>106</v>
+        <v>133</v>
       </c>
       <c r="D347" t="s">
-        <v>928</v>
+        <v>996</v>
+      </c>
+      <c r="E347" t="s">
+        <v>152</v>
+      </c>
+      <c r="F347" t="s">
+        <v>141</v>
       </c>
       <c r="H347" t="s">
         <v>119</v>
@@ -13697,13 +13733,19 @@
     </row>
     <row r="348" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
-        <v>972</v>
+        <v>1005</v>
       </c>
       <c r="B348" t="s">
-        <v>970</v>
+        <v>133</v>
       </c>
       <c r="D348" t="s">
-        <v>961</v>
+        <v>997</v>
+      </c>
+      <c r="E348" t="s">
+        <v>152</v>
+      </c>
+      <c r="F348" t="s">
+        <v>141</v>
       </c>
       <c r="H348" t="s">
         <v>119</v>
@@ -13714,13 +13756,19 @@
     </row>
     <row r="349" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
-        <v>971</v>
+        <v>1006</v>
       </c>
       <c r="B349" t="s">
-        <v>970</v>
+        <v>133</v>
       </c>
       <c r="D349" t="s">
-        <v>962</v>
+        <v>998</v>
+      </c>
+      <c r="E349" t="s">
+        <v>152</v>
+      </c>
+      <c r="F349" t="s">
+        <v>141</v>
       </c>
       <c r="H349" t="s">
         <v>119</v>
@@ -13731,13 +13779,13 @@
     </row>
     <row r="350" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
-        <v>973</v>
+        <v>925</v>
       </c>
       <c r="B350" t="s">
-        <v>970</v>
+        <v>106</v>
       </c>
       <c r="D350" t="s">
-        <v>963</v>
+        <v>926</v>
       </c>
       <c r="H350" t="s">
         <v>119</v>
@@ -13748,13 +13796,13 @@
     </row>
     <row r="351" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
-        <v>974</v>
+        <v>927</v>
       </c>
       <c r="B351" t="s">
-        <v>970</v>
+        <v>106</v>
       </c>
       <c r="D351" t="s">
-        <v>964</v>
+        <v>928</v>
       </c>
       <c r="H351" t="s">
         <v>119</v>
@@ -13765,13 +13813,13 @@
     </row>
     <row r="352" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
-        <v>975</v>
+        <v>972</v>
       </c>
       <c r="B352" t="s">
         <v>970</v>
       </c>
       <c r="D352" t="s">
-        <v>965</v>
+        <v>961</v>
       </c>
       <c r="H352" t="s">
         <v>119</v>
@@ -13782,13 +13830,13 @@
     </row>
     <row r="353" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
-        <v>976</v>
+        <v>971</v>
       </c>
       <c r="B353" t="s">
         <v>970</v>
       </c>
       <c r="D353" t="s">
-        <v>966</v>
+        <v>962</v>
       </c>
       <c r="H353" t="s">
         <v>119</v>
@@ -13799,13 +13847,13 @@
     </row>
     <row r="354" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
-        <v>977</v>
+        <v>973</v>
       </c>
       <c r="B354" t="s">
         <v>970</v>
       </c>
       <c r="D354" t="s">
-        <v>967</v>
+        <v>963</v>
       </c>
       <c r="H354" t="s">
         <v>119</v>
@@ -13816,13 +13864,13 @@
     </row>
     <row r="355" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
-        <v>978</v>
+        <v>974</v>
       </c>
       <c r="B355" t="s">
         <v>970</v>
       </c>
       <c r="D355" t="s">
-        <v>968</v>
+        <v>964</v>
       </c>
       <c r="H355" t="s">
         <v>119</v>
@@ -13833,13 +13881,13 @@
     </row>
     <row r="356" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
-        <v>979</v>
+        <v>975</v>
       </c>
       <c r="B356" t="s">
         <v>970</v>
       </c>
       <c r="D356" t="s">
-        <v>969</v>
+        <v>965</v>
       </c>
       <c r="H356" t="s">
         <v>119</v>
@@ -13850,104 +13898,172 @@
     </row>
     <row r="357" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
-        <v>980</v>
+        <v>976</v>
       </c>
       <c r="B357" t="s">
-        <v>106</v>
+        <v>970</v>
       </c>
       <c r="D357" t="s">
-        <v>981</v>
-      </c>
-      <c r="E357" t="s">
-        <v>152</v>
-      </c>
-      <c r="F357" t="s">
-        <v>982</v>
+        <v>966</v>
       </c>
       <c r="H357" t="s">
+        <v>119</v>
+      </c>
+      <c r="I357" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="358" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
-        <v>983</v>
+        <v>977</v>
       </c>
       <c r="B358" t="s">
-        <v>106</v>
+        <v>970</v>
       </c>
       <c r="D358" t="s">
-        <v>984</v>
-      </c>
-      <c r="E358" t="s">
-        <v>152</v>
-      </c>
-      <c r="F358" t="s">
-        <v>982</v>
+        <v>967</v>
       </c>
       <c r="H358" t="s">
+        <v>119</v>
+      </c>
+      <c r="I358" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="359" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
-        <v>985</v>
+        <v>978</v>
       </c>
       <c r="B359" t="s">
-        <v>106</v>
+        <v>970</v>
       </c>
       <c r="D359" t="s">
-        <v>986</v>
-      </c>
-      <c r="E359" t="s">
-        <v>152</v>
-      </c>
-      <c r="F359" t="s">
-        <v>982</v>
+        <v>968</v>
       </c>
       <c r="H359" t="s">
+        <v>119</v>
+      </c>
+      <c r="I359" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="360" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
-        <v>987</v>
+        <v>979</v>
       </c>
       <c r="B360" t="s">
-        <v>106</v>
+        <v>970</v>
       </c>
       <c r="D360" t="s">
-        <v>988</v>
-      </c>
-      <c r="E360" t="s">
-        <v>152</v>
-      </c>
-      <c r="F360" t="s">
-        <v>982</v>
+        <v>969</v>
       </c>
       <c r="H360" t="s">
+        <v>119</v>
+      </c>
+      <c r="I360" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="361" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
+        <v>980</v>
+      </c>
+      <c r="B361" t="s">
+        <v>106</v>
+      </c>
+      <c r="D361" t="s">
+        <v>981</v>
+      </c>
+      <c r="E361" t="s">
+        <v>152</v>
+      </c>
+      <c r="F361" t="s">
+        <v>982</v>
+      </c>
+      <c r="H361" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="362" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A362" t="s">
+        <v>983</v>
+      </c>
+      <c r="B362" t="s">
+        <v>106</v>
+      </c>
+      <c r="D362" t="s">
+        <v>984</v>
+      </c>
+      <c r="E362" t="s">
+        <v>152</v>
+      </c>
+      <c r="F362" t="s">
+        <v>982</v>
+      </c>
+      <c r="H362" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="363" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A363" t="s">
+        <v>985</v>
+      </c>
+      <c r="B363" t="s">
+        <v>106</v>
+      </c>
+      <c r="D363" t="s">
+        <v>986</v>
+      </c>
+      <c r="E363" t="s">
+        <v>152</v>
+      </c>
+      <c r="F363" t="s">
+        <v>982</v>
+      </c>
+      <c r="H363" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="364" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A364" t="s">
+        <v>987</v>
+      </c>
+      <c r="B364" t="s">
+        <v>106</v>
+      </c>
+      <c r="D364" t="s">
+        <v>988</v>
+      </c>
+      <c r="E364" t="s">
+        <v>152</v>
+      </c>
+      <c r="F364" t="s">
+        <v>982</v>
+      </c>
+      <c r="H364" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="365" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A365" t="s">
         <v>989</v>
       </c>
-      <c r="B361" t="s">
-        <v>106</v>
-      </c>
-      <c r="D361" t="s">
+      <c r="B365" t="s">
+        <v>106</v>
+      </c>
+      <c r="D365" t="s">
         <v>990</v>
       </c>
-      <c r="E361" t="s">
-        <v>152</v>
-      </c>
-      <c r="F361" t="s">
-        <v>141</v>
-      </c>
-      <c r="H361" t="s">
-        <v>119</v>
-      </c>
-      <c r="I361" t="s">
+      <c r="E365" t="s">
+        <v>152</v>
+      </c>
+      <c r="F365" t="s">
+        <v>141</v>
+      </c>
+      <c r="H365" t="s">
+        <v>119</v>
+      </c>
+      <c r="I365" t="s">
         <v>119</v>
       </c>
     </row>
@@ -13957,7 +14073,7 @@
       <sortCondition ref="B1:B341"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="J16:J21 J86:J91 J105 J117 J149 J214 E2:E345">
+  <conditionalFormatting sqref="J16:J21 J86:J91 J105 J117 J149 J214 E2:E349">
     <cfRule type="containsText" dxfId="19" priority="90" operator="containsText" text="no">
       <formula>NOT(ISERROR(SEARCH("no",E2)))</formula>
     </cfRule>
@@ -13965,7 +14081,7 @@
       <formula>NOT(ISERROR(SEARCH("yes",E2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E345">
+  <conditionalFormatting sqref="E2:E349">
     <cfRule type="containsText" dxfId="17" priority="87" operator="containsText" text="no">
       <formula>NOT(ISERROR(SEARCH("no",E2)))</formula>
     </cfRule>
@@ -13973,35 +14089,35 @@
       <formula>NOT(ISERROR(SEARCH("TBD",E2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E361">
+  <conditionalFormatting sqref="E365">
     <cfRule type="containsText" dxfId="15" priority="1" operator="containsText" text="no">
+      <formula>NOT(ISERROR(SEARCH("no",E365)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="14" priority="2" operator="containsText" text="TBD">
+      <formula>NOT(ISERROR(SEARCH("TBD",E365)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="13" priority="3" operator="containsText" text="no">
+      <formula>NOT(ISERROR(SEARCH("no",E365)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="12" priority="4" operator="containsText" text="yes">
+      <formula>NOT(ISERROR(SEARCH("yes",E365)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E361:F364">
+    <cfRule type="containsText" dxfId="11" priority="5" operator="containsText" text="no">
       <formula>NOT(ISERROR(SEARCH("no",E361)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="2" operator="containsText" text="TBD">
+    <cfRule type="containsText" dxfId="10" priority="6" operator="containsText" text="TBD">
       <formula>NOT(ISERROR(SEARCH("TBD",E361)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="3" operator="containsText" text="no">
+    <cfRule type="containsText" dxfId="9" priority="7" operator="containsText" text="no">
       <formula>NOT(ISERROR(SEARCH("no",E361)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="4" operator="containsText" text="yes">
+    <cfRule type="containsText" dxfId="8" priority="8" operator="containsText" text="yes">
       <formula>NOT(ISERROR(SEARCH("yes",E361)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E357:F360">
-    <cfRule type="containsText" dxfId="11" priority="5" operator="containsText" text="no">
-      <formula>NOT(ISERROR(SEARCH("no",E357)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="6" operator="containsText" text="TBD">
-      <formula>NOT(ISERROR(SEARCH("TBD",E357)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="7" operator="containsText" text="no">
-      <formula>NOT(ISERROR(SEARCH("no",E357)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="8" operator="containsText" text="yes">
-      <formula>NOT(ISERROR(SEARCH("yes",E357)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H2:I356">
+  <conditionalFormatting sqref="H2:I360">
     <cfRule type="containsText" dxfId="7" priority="9" operator="containsText" text="no">
       <formula>NOT(ISERROR(SEARCH("no",H2)))</formula>
     </cfRule>

</xml_diff>